<commit_message>
补充 情种(Klimter HopelessRomanticTrait) 的百度网盘链接
</commit_message>
<xml_diff>
--- a/content/作品信息.xlsx
+++ b/content/作品信息.xlsx
@@ -618,7 +618,11 @@
           <t>images/klimter-hopelessromantictrait.png</t>
         </is>
       </c>
-      <c r="K4" s="10" t="str"/>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>链接: https://pan.baidu.com/s/1ZAvlvcY8HZPdyl0gcs21dg 提取码: c22c</t>
+        </is>
+      </c>
       <c r="L4" s="12" t="inlineStr">
         <is>
           <t>人物特征</t>

</xml_diff>

<commit_message>
修正 Klimter - ParentalTrait（称职父母）发布日期为 2026-08-19
</commit_message>
<xml_diff>
--- a/content/作品信息.xlsx
+++ b/content/作品信息.xlsx
@@ -2341,10 +2341,10 @@
         </is>
       </c>
       <c r="F34" s="16" t="n">
-        <v>46250</v>
+        <v>46253</v>
       </c>
       <c r="G34" s="16" t="n">
-        <v>46250</v>
+        <v>46253</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>

</xml_diff>